<commit_message>
refactor(schema): move field parsing options into parser
</commit_message>
<xml_diff>
--- a/examples/showcase/data/Battle.xlsx
+++ b/examples/showcase/data/Battle.xlsx
@@ -52,7 +52,7 @@
     <t>@schema</t>
   </si>
   <si>
-    <t>139bd0c7b236a4cf</t>
+    <t>70fc913f3e9b878f</t>
   </si>
   <si>
     <t>#name</t>
@@ -118,7 +118,7 @@
     <t>required</t>
   </si>
   <si>
-    <t>required;separator=,;parser=tuple</t>
+    <t>required;parser=tuple</t>
   </si>
   <si>
     <t>optional;range=1..100</t>
@@ -697,7 +697,7 @@
     <t>Character</t>
   </si>
   <si>
-    <t>d2c006329eed6eb3</t>
+    <t>996fe1623cec07ee</t>
   </si>
   <si>
     <t>rarity</t>
@@ -727,9 +727,6 @@
     <t>list&lt;ref&lt;Item.id&gt;&gt;</t>
   </si>
   <si>
-    <t>required;separator=,;prefix=[;suffix=]</t>
-  </si>
-  <si>
     <t>4001</t>
   </si>
   <si>
@@ -994,7 +991,7 @@
     <t>list</t>
   </si>
   <si>
-    <t>3c9049eb1a8a8b3e</t>
+    <t>e92c79afa1e2e40b</t>
   </si>
   <si>
     <t>character_id</t>
@@ -1015,7 +1012,7 @@
     <t>Buff</t>
   </si>
   <si>
-    <t>5664e2665d4d2fff</t>
+    <t>ab300d6757967f84</t>
   </si>
   <si>
     <t>duration</t>
@@ -1030,6 +1027,9 @@
     <t>list&lt;struct&lt;StatModifier&gt;&gt;</t>
   </si>
   <si>
+    <t>required;parser=json</t>
+  </si>
+  <si>
     <t>6001</t>
   </si>
   <si>
@@ -1213,7 +1213,7 @@
     <t>DropGroup</t>
   </si>
   <si>
-    <t>198e3bc14f1ae42b</t>
+    <t>ddc8f184c6f4ca0b</t>
   </si>
   <si>
     <t>7001</t>
@@ -1339,7 +1339,7 @@
     <t>DropEntry</t>
   </si>
   <si>
-    <t>430779b9896d046d</t>
+    <t>38e6bc608bd50c74</t>
   </si>
   <si>
     <t>group_id</t>
@@ -1438,7 +1438,7 @@
     <t>Monster</t>
   </si>
   <si>
-    <t>528a6db4e291242f</t>
+    <t>3f0a6c4362bc5a57</t>
   </si>
   <si>
     <t>level</t>
@@ -2239,7 +2239,7 @@
     <t>Stage</t>
   </si>
   <si>
-    <t>ff19dbdf0f0e4b94</t>
+    <t>bede35fc90989759</t>
   </si>
   <si>
     <t>monster_ids</t>
@@ -2740,7 +2740,7 @@
     <t>StageReward</t>
   </si>
   <si>
-    <t>88182c561a3498ab</t>
+    <t>0c97ec70735264e3</t>
   </si>
   <si>
     <t>stage_id</t>
@@ -2809,7 +2809,7 @@
     <t>Dungeon</t>
   </si>
   <si>
-    <t>eee9bc33ced1d705</t>
+    <t>b0a9bd963cf8bc87</t>
   </si>
   <si>
     <t>stage_ids</t>
@@ -4318,7 +4318,7 @@
         <v>30</v>
       </c>
       <c r="D11" t="s">
-        <v>234</v>
+        <v>30</v>
       </c>
       <c r="E11" t="s">
         <v>31</v>
@@ -4643,7 +4643,7 @@
         <v>30</v>
       </c>
       <c r="G11" t="s">
-        <v>234</v>
+        <v>30</v>
       </c>
       <c r="H11" t="s">
         <v>31</v>
@@ -4656,36 +4656,36 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
+        <v>234</v>
+      </c>
+      <c r="B13" t="s">
         <v>235</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>236</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>237</v>
-      </c>
-      <c r="D13" t="s">
-        <v>238</v>
       </c>
       <c r="E13" t="s">
         <v>109</v>
       </c>
       <c r="F13" t="s">
+        <v>238</v>
+      </c>
+      <c r="G13" t="s">
         <v>239</v>
-      </c>
-      <c r="G13" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
+        <v>240</v>
+      </c>
+      <c r="B14" t="s">
         <v>241</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>242</v>
-      </c>
-      <c r="C14" t="s">
-        <v>243</v>
       </c>
       <c r="D14" t="s">
         <v>43</v>
@@ -4694,21 +4694,21 @@
         <v>115</v>
       </c>
       <c r="F14" t="s">
+        <v>243</v>
+      </c>
+      <c r="G14" t="s">
         <v>244</v>
-      </c>
-      <c r="G14" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
+        <v>245</v>
+      </c>
+      <c r="B15" t="s">
         <v>246</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>247</v>
-      </c>
-      <c r="C15" t="s">
-        <v>248</v>
       </c>
       <c r="D15" t="s">
         <v>57</v>
@@ -4717,21 +4717,21 @@
         <v>121</v>
       </c>
       <c r="F15" t="s">
+        <v>248</v>
+      </c>
+      <c r="G15" t="s">
         <v>249</v>
-      </c>
-      <c r="G15" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" t="s">
+        <v>250</v>
+      </c>
+      <c r="B16" t="s">
         <v>251</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>252</v>
-      </c>
-      <c r="C16" t="s">
-        <v>253</v>
       </c>
       <c r="D16" t="s">
         <v>63</v>
@@ -4740,21 +4740,21 @@
         <v>127</v>
       </c>
       <c r="F16" t="s">
+        <v>253</v>
+      </c>
+      <c r="G16" t="s">
         <v>254</v>
-      </c>
-      <c r="G16" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" t="s">
+        <v>255</v>
+      </c>
+      <c r="B17" t="s">
         <v>256</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>257</v>
-      </c>
-      <c r="C17" t="s">
-        <v>258</v>
       </c>
       <c r="D17" t="s">
         <v>69</v>
@@ -4763,21 +4763,21 @@
         <v>133</v>
       </c>
       <c r="F17" t="s">
+        <v>258</v>
+      </c>
+      <c r="G17" t="s">
         <v>259</v>
-      </c>
-      <c r="G17" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" t="s">
+        <v>260</v>
+      </c>
+      <c r="B18" t="s">
         <v>261</v>
       </c>
-      <c r="B18" t="s">
-        <v>262</v>
-      </c>
       <c r="C18" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D18" t="s">
         <v>77</v>
@@ -4786,21 +4786,21 @@
         <v>139</v>
       </c>
       <c r="F18" t="s">
+        <v>262</v>
+      </c>
+      <c r="G18" t="s">
         <v>263</v>
-      </c>
-      <c r="G18" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="19" spans="1:7">
       <c r="A19" t="s">
+        <v>264</v>
+      </c>
+      <c r="B19" t="s">
         <v>265</v>
       </c>
-      <c r="B19" t="s">
-        <v>266</v>
-      </c>
       <c r="C19" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D19" t="s">
         <v>83</v>
@@ -4809,21 +4809,21 @@
         <v>145</v>
       </c>
       <c r="F19" t="s">
+        <v>266</v>
+      </c>
+      <c r="G19" t="s">
         <v>267</v>
-      </c>
-      <c r="G19" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" t="s">
+        <v>268</v>
+      </c>
+      <c r="B20" t="s">
         <v>269</v>
       </c>
-      <c r="B20" t="s">
-        <v>270</v>
-      </c>
       <c r="C20" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D20" t="s">
         <v>89</v>
@@ -4832,21 +4832,21 @@
         <v>151</v>
       </c>
       <c r="F20" t="s">
+        <v>270</v>
+      </c>
+      <c r="G20" t="s">
         <v>271</v>
-      </c>
-      <c r="G20" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" t="s">
+        <v>272</v>
+      </c>
+      <c r="B21" t="s">
         <v>273</v>
       </c>
-      <c r="B21" t="s">
-        <v>274</v>
-      </c>
       <c r="C21" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D21" t="s">
         <v>95</v>
@@ -4855,21 +4855,21 @@
         <v>157</v>
       </c>
       <c r="F21" t="s">
+        <v>274</v>
+      </c>
+      <c r="G21" t="s">
         <v>275</v>
-      </c>
-      <c r="G21" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" t="s">
+        <v>276</v>
+      </c>
+      <c r="B22" t="s">
         <v>277</v>
       </c>
-      <c r="B22" t="s">
-        <v>278</v>
-      </c>
       <c r="C22" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D22" t="s">
         <v>101</v>
@@ -4878,21 +4878,21 @@
         <v>163</v>
       </c>
       <c r="F22" t="s">
+        <v>278</v>
+      </c>
+      <c r="G22" t="s">
         <v>279</v>
-      </c>
-      <c r="G22" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" t="s">
+        <v>280</v>
+      </c>
+      <c r="B23" t="s">
         <v>281</v>
       </c>
-      <c r="B23" t="s">
-        <v>282</v>
-      </c>
       <c r="C23" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D23" t="s">
         <v>107</v>
@@ -4901,21 +4901,21 @@
         <v>169</v>
       </c>
       <c r="F23" t="s">
+        <v>282</v>
+      </c>
+      <c r="G23" t="s">
         <v>283</v>
-      </c>
-      <c r="G23" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="24" spans="1:7">
       <c r="A24" t="s">
+        <v>284</v>
+      </c>
+      <c r="B24" t="s">
         <v>285</v>
       </c>
-      <c r="B24" t="s">
-        <v>286</v>
-      </c>
       <c r="C24" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D24" t="s">
         <v>113</v>
@@ -4924,21 +4924,21 @@
         <v>175</v>
       </c>
       <c r="F24" t="s">
+        <v>286</v>
+      </c>
+      <c r="G24" t="s">
         <v>287</v>
-      </c>
-      <c r="G24" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="25" spans="1:7">
       <c r="A25" t="s">
+        <v>288</v>
+      </c>
+      <c r="B25" t="s">
         <v>289</v>
       </c>
-      <c r="B25" t="s">
-        <v>290</v>
-      </c>
       <c r="C25" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D25" t="s">
         <v>119</v>
@@ -4947,21 +4947,21 @@
         <v>181</v>
       </c>
       <c r="F25" t="s">
+        <v>290</v>
+      </c>
+      <c r="G25" t="s">
         <v>291</v>
-      </c>
-      <c r="G25" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="26" spans="1:7">
       <c r="A26" t="s">
+        <v>292</v>
+      </c>
+      <c r="B26" t="s">
         <v>293</v>
       </c>
-      <c r="B26" t="s">
-        <v>294</v>
-      </c>
       <c r="C26" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D26" t="s">
         <v>125</v>
@@ -4970,21 +4970,21 @@
         <v>187</v>
       </c>
       <c r="F26" t="s">
+        <v>294</v>
+      </c>
+      <c r="G26" t="s">
         <v>295</v>
-      </c>
-      <c r="G26" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="27" spans="1:7">
       <c r="A27" t="s">
+        <v>296</v>
+      </c>
+      <c r="B27" t="s">
         <v>297</v>
       </c>
-      <c r="B27" t="s">
-        <v>298</v>
-      </c>
       <c r="C27" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D27" t="s">
         <v>131</v>
@@ -4993,21 +4993,21 @@
         <v>193</v>
       </c>
       <c r="F27" t="s">
+        <v>298</v>
+      </c>
+      <c r="G27" t="s">
         <v>299</v>
-      </c>
-      <c r="G27" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="28" spans="1:7">
       <c r="A28" t="s">
+        <v>300</v>
+      </c>
+      <c r="B28" t="s">
         <v>301</v>
       </c>
-      <c r="B28" t="s">
-        <v>302</v>
-      </c>
       <c r="C28" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D28" t="s">
         <v>137</v>
@@ -5016,21 +5016,21 @@
         <v>199</v>
       </c>
       <c r="F28" t="s">
+        <v>302</v>
+      </c>
+      <c r="G28" t="s">
         <v>303</v>
-      </c>
-      <c r="G28" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="29" spans="1:7">
       <c r="A29" t="s">
+        <v>304</v>
+      </c>
+      <c r="B29" t="s">
         <v>305</v>
       </c>
-      <c r="B29" t="s">
-        <v>306</v>
-      </c>
       <c r="C29" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D29" t="s">
         <v>143</v>
@@ -5039,21 +5039,21 @@
         <v>205</v>
       </c>
       <c r="F29" t="s">
+        <v>306</v>
+      </c>
+      <c r="G29" t="s">
         <v>307</v>
-      </c>
-      <c r="G29" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="30" spans="1:7">
       <c r="A30" t="s">
+        <v>308</v>
+      </c>
+      <c r="B30" t="s">
         <v>309</v>
       </c>
-      <c r="B30" t="s">
-        <v>310</v>
-      </c>
       <c r="C30" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D30" t="s">
         <v>149</v>
@@ -5062,21 +5062,21 @@
         <v>211</v>
       </c>
       <c r="F30" t="s">
+        <v>310</v>
+      </c>
+      <c r="G30" t="s">
         <v>311</v>
-      </c>
-      <c r="G30" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="31" spans="1:7">
       <c r="A31" t="s">
+        <v>312</v>
+      </c>
+      <c r="B31" t="s">
         <v>313</v>
       </c>
-      <c r="B31" t="s">
-        <v>314</v>
-      </c>
       <c r="C31" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D31" t="s">
         <v>155</v>
@@ -5085,21 +5085,21 @@
         <v>217</v>
       </c>
       <c r="F31" t="s">
+        <v>314</v>
+      </c>
+      <c r="G31" t="s">
         <v>315</v>
-      </c>
-      <c r="G31" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="32" spans="1:7">
       <c r="A32" t="s">
+        <v>316</v>
+      </c>
+      <c r="B32" t="s">
         <v>317</v>
       </c>
-      <c r="B32" t="s">
-        <v>318</v>
-      </c>
       <c r="C32" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D32" t="s">
         <v>161</v>
@@ -5108,10 +5108,10 @@
         <v>38</v>
       </c>
       <c r="F32" t="s">
+        <v>318</v>
+      </c>
+      <c r="G32" t="s">
         <v>319</v>
-      </c>
-      <c r="G32" t="s">
-        <v>320</v>
       </c>
     </row>
   </sheetData>
@@ -5129,7 +5129,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -5137,7 +5137,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -5158,7 +5158,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -5166,13 +5166,13 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
+        <v>323</v>
+      </c>
+      <c r="C7" t="s">
         <v>324</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>325</v>
-      </c>
-      <c r="D7" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -5180,13 +5180,13 @@
         <v>18</v>
       </c>
       <c r="B8" t="s">
+        <v>323</v>
+      </c>
+      <c r="C8" t="s">
         <v>324</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>325</v>
-      </c>
-      <c r="D8" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -5194,7 +5194,7 @@
         <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C9" t="s">
         <v>232</v>
@@ -5238,18 +5238,18 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B13" t="s">
         <v>109</v>
       </c>
       <c r="C13" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B14" t="s">
         <v>115</v>
@@ -5260,7 +5260,7 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B15" t="s">
         <v>121</v>
@@ -5271,18 +5271,18 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B16" t="s">
         <v>115</v>
       </c>
       <c r="C16" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B17" t="s">
         <v>121</v>
@@ -5293,7 +5293,7 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B18" t="s">
         <v>127</v>
@@ -5304,18 +5304,18 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B19" t="s">
         <v>121</v>
       </c>
       <c r="C19" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B20" t="s">
         <v>127</v>
@@ -5326,7 +5326,7 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B21" t="s">
         <v>133</v>
@@ -5337,18 +5337,18 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B22" t="s">
         <v>127</v>
       </c>
       <c r="C22" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B23" t="s">
         <v>133</v>
@@ -5359,7 +5359,7 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B24" t="s">
         <v>139</v>
@@ -5370,18 +5370,18 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B25" t="s">
         <v>133</v>
       </c>
       <c r="C25" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B26" t="s">
         <v>139</v>
@@ -5392,7 +5392,7 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B27" t="s">
         <v>145</v>
@@ -5403,18 +5403,18 @@
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B28" t="s">
         <v>139</v>
       </c>
       <c r="C28" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B29" t="s">
         <v>145</v>
@@ -5425,7 +5425,7 @@
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B30" t="s">
         <v>151</v>
@@ -5436,18 +5436,18 @@
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B31" t="s">
         <v>145</v>
       </c>
       <c r="C31" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B32" t="s">
         <v>151</v>
@@ -5458,7 +5458,7 @@
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B33" t="s">
         <v>157</v>
@@ -5469,18 +5469,18 @@
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B34" t="s">
         <v>151</v>
       </c>
       <c r="C34" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B35" t="s">
         <v>157</v>
@@ -5491,7 +5491,7 @@
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B36" t="s">
         <v>163</v>
@@ -5502,18 +5502,18 @@
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B37" t="s">
         <v>157</v>
       </c>
       <c r="C37" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B38" t="s">
         <v>163</v>
@@ -5524,7 +5524,7 @@
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B39" t="s">
         <v>169</v>
@@ -5535,18 +5535,18 @@
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B40" t="s">
         <v>163</v>
       </c>
       <c r="C40" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B41" t="s">
         <v>169</v>
@@ -5557,7 +5557,7 @@
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B42" t="s">
         <v>175</v>
@@ -5568,18 +5568,18 @@
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B43" t="s">
         <v>169</v>
       </c>
       <c r="C43" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B44" t="s">
         <v>175</v>
@@ -5590,7 +5590,7 @@
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B45" t="s">
         <v>181</v>
@@ -5601,18 +5601,18 @@
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B46" t="s">
         <v>175</v>
       </c>
       <c r="C46" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B47" t="s">
         <v>181</v>
@@ -5623,7 +5623,7 @@
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B48" t="s">
         <v>187</v>
@@ -5634,18 +5634,18 @@
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B49" t="s">
         <v>181</v>
       </c>
       <c r="C49" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B50" t="s">
         <v>187</v>
@@ -5656,7 +5656,7 @@
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B51" t="s">
         <v>193</v>
@@ -5667,18 +5667,18 @@
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B52" t="s">
         <v>187</v>
       </c>
       <c r="C52" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B53" t="s">
         <v>193</v>
@@ -5689,7 +5689,7 @@
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B54" t="s">
         <v>199</v>
@@ -5700,18 +5700,18 @@
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B55" t="s">
         <v>193</v>
       </c>
       <c r="C55" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B56" t="s">
         <v>199</v>
@@ -5722,7 +5722,7 @@
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B57" t="s">
         <v>205</v>
@@ -5733,18 +5733,18 @@
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B58" t="s">
         <v>199</v>
       </c>
       <c r="C58" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B59" t="s">
         <v>205</v>
@@ -5755,7 +5755,7 @@
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B60" t="s">
         <v>211</v>
@@ -5766,18 +5766,18 @@
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B61" t="s">
         <v>205</v>
       </c>
       <c r="C61" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B62" t="s">
         <v>211</v>
@@ -5788,7 +5788,7 @@
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B63" t="s">
         <v>217</v>
@@ -5799,18 +5799,18 @@
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B64" t="s">
         <v>211</v>
       </c>
       <c r="C64" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B65" t="s">
         <v>217</v>
@@ -5821,7 +5821,7 @@
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B66" t="s">
         <v>38</v>
@@ -5832,18 +5832,18 @@
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B67" t="s">
         <v>217</v>
       </c>
       <c r="C67" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B68" t="s">
         <v>38</v>
@@ -5854,7 +5854,7 @@
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B69" t="s">
         <v>46</v>
@@ -5865,18 +5865,18 @@
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B70" t="s">
         <v>38</v>
       </c>
       <c r="C70" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B71" t="s">
         <v>46</v>
@@ -5887,7 +5887,7 @@
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B72" t="s">
         <v>52</v>
@@ -5911,7 +5911,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -5943,7 +5943,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -5957,10 +5957,10 @@
         <v>11</v>
       </c>
       <c r="D7" t="s">
+        <v>330</v>
+      </c>
+      <c r="E7" t="s">
         <v>331</v>
-      </c>
-      <c r="E7" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -5974,10 +5974,10 @@
         <v>11</v>
       </c>
       <c r="D8" t="s">
+        <v>330</v>
+      </c>
+      <c r="E8" t="s">
         <v>331</v>
-      </c>
-      <c r="E8" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -5991,10 +5991,10 @@
         <v>21</v>
       </c>
       <c r="D9" t="s">
+        <v>332</v>
+      </c>
+      <c r="E9" t="s">
         <v>333</v>
-      </c>
-      <c r="E9" t="s">
-        <v>334</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -6028,7 +6028,7 @@
         <v>30</v>
       </c>
       <c r="E11" t="s">
-        <v>234</v>
+        <v>334</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -6609,7 +6609,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -6690,7 +6690,7 @@
         <v>20</v>
       </c>
       <c r="F9" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -6743,7 +6743,7 @@
         <v>397</v>
       </c>
       <c r="B13" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C13" t="s">
         <v>448</v>
@@ -6760,7 +6760,7 @@
         <v>397</v>
       </c>
       <c r="B14" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C14" t="s">
         <v>449</v>
@@ -6794,7 +6794,7 @@
         <v>399</v>
       </c>
       <c r="B16" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C16" t="s">
         <v>449</v>
@@ -6811,7 +6811,7 @@
         <v>399</v>
       </c>
       <c r="B17" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C17" t="s">
         <v>450</v>
@@ -6845,7 +6845,7 @@
         <v>401</v>
       </c>
       <c r="B19" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C19" t="s">
         <v>450</v>
@@ -6862,7 +6862,7 @@
         <v>401</v>
       </c>
       <c r="B20" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C20" t="s">
         <v>451</v>
@@ -6896,7 +6896,7 @@
         <v>403</v>
       </c>
       <c r="B22" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C22" t="s">
         <v>451</v>
@@ -6913,7 +6913,7 @@
         <v>403</v>
       </c>
       <c r="B23" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C23" t="s">
         <v>452</v>
@@ -6947,7 +6947,7 @@
         <v>405</v>
       </c>
       <c r="B25" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C25" t="s">
         <v>452</v>
@@ -6964,7 +6964,7 @@
         <v>405</v>
       </c>
       <c r="B26" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C26" t="s">
         <v>453</v>
@@ -6998,7 +6998,7 @@
         <v>407</v>
       </c>
       <c r="B28" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C28" t="s">
         <v>453</v>
@@ -7015,7 +7015,7 @@
         <v>407</v>
       </c>
       <c r="B29" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C29" t="s">
         <v>454</v>
@@ -7049,7 +7049,7 @@
         <v>409</v>
       </c>
       <c r="B31" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C31" t="s">
         <v>454</v>
@@ -7066,7 +7066,7 @@
         <v>409</v>
       </c>
       <c r="B32" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C32" t="s">
         <v>455</v>
@@ -7100,7 +7100,7 @@
         <v>411</v>
       </c>
       <c r="B34" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C34" t="s">
         <v>455</v>
@@ -7117,7 +7117,7 @@
         <v>411</v>
       </c>
       <c r="B35" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C35" t="s">
         <v>456</v>
@@ -7151,7 +7151,7 @@
         <v>413</v>
       </c>
       <c r="B37" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C37" t="s">
         <v>456</v>
@@ -7168,7 +7168,7 @@
         <v>413</v>
       </c>
       <c r="B38" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C38" t="s">
         <v>457</v>
@@ -7202,7 +7202,7 @@
         <v>415</v>
       </c>
       <c r="B40" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C40" t="s">
         <v>457</v>
@@ -7219,7 +7219,7 @@
         <v>415</v>
       </c>
       <c r="B41" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C41" t="s">
         <v>458</v>
@@ -7253,7 +7253,7 @@
         <v>417</v>
       </c>
       <c r="B43" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C43" t="s">
         <v>458</v>
@@ -7270,7 +7270,7 @@
         <v>417</v>
       </c>
       <c r="B44" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C44" t="s">
         <v>459</v>
@@ -7304,7 +7304,7 @@
         <v>419</v>
       </c>
       <c r="B46" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C46" t="s">
         <v>459</v>
@@ -7321,7 +7321,7 @@
         <v>419</v>
       </c>
       <c r="B47" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C47" t="s">
         <v>460</v>
@@ -7355,7 +7355,7 @@
         <v>421</v>
       </c>
       <c r="B49" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C49" t="s">
         <v>460</v>
@@ -7372,7 +7372,7 @@
         <v>421</v>
       </c>
       <c r="B50" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C50" t="s">
         <v>461</v>
@@ -7406,7 +7406,7 @@
         <v>423</v>
       </c>
       <c r="B52" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C52" t="s">
         <v>461</v>
@@ -7423,7 +7423,7 @@
         <v>423</v>
       </c>
       <c r="B53" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C53" t="s">
         <v>462</v>
@@ -7457,7 +7457,7 @@
         <v>425</v>
       </c>
       <c r="B55" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C55" t="s">
         <v>462</v>
@@ -7474,7 +7474,7 @@
         <v>425</v>
       </c>
       <c r="B56" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C56" t="s">
         <v>463</v>
@@ -7508,7 +7508,7 @@
         <v>427</v>
       </c>
       <c r="B58" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C58" t="s">
         <v>463</v>
@@ -7525,7 +7525,7 @@
         <v>427</v>
       </c>
       <c r="B59" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C59" t="s">
         <v>464</v>
@@ -7559,7 +7559,7 @@
         <v>429</v>
       </c>
       <c r="B61" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C61" t="s">
         <v>464</v>
@@ -7576,7 +7576,7 @@
         <v>429</v>
       </c>
       <c r="B62" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C62" t="s">
         <v>465</v>
@@ -7610,7 +7610,7 @@
         <v>431</v>
       </c>
       <c r="B64" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C64" t="s">
         <v>465</v>
@@ -7627,7 +7627,7 @@
         <v>431</v>
       </c>
       <c r="B65" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C65" t="s">
         <v>466</v>
@@ -7661,7 +7661,7 @@
         <v>433</v>
       </c>
       <c r="B67" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C67" t="s">
         <v>466</v>
@@ -7678,7 +7678,7 @@
         <v>433</v>
       </c>
       <c r="B68" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C68" t="s">
         <v>467</v>
@@ -7712,7 +7712,7 @@
         <v>435</v>
       </c>
       <c r="B70" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C70" t="s">
         <v>467</v>
@@ -7729,7 +7729,7 @@
         <v>435</v>
       </c>
       <c r="B71" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C71" t="s">
         <v>468</v>
@@ -7936,7 +7936,7 @@
         <v>475</v>
       </c>
       <c r="C13" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="D13" t="s">
         <v>48</v>
@@ -8725,7 +8725,7 @@
         <v>397</v>
       </c>
       <c r="F52" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="53" spans="1:6">
@@ -8745,7 +8745,7 @@
         <v>399</v>
       </c>
       <c r="F53" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="54" spans="1:6">
@@ -8765,7 +8765,7 @@
         <v>401</v>
       </c>
       <c r="F54" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="55" spans="1:6">
@@ -8785,7 +8785,7 @@
         <v>403</v>
       </c>
       <c r="F55" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="56" spans="1:6">
@@ -8805,7 +8805,7 @@
         <v>405</v>
       </c>
       <c r="F56" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="57" spans="1:6">
@@ -8825,7 +8825,7 @@
         <v>407</v>
       </c>
       <c r="F57" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="58" spans="1:6">
@@ -9516,7 +9516,7 @@
         <v>736</v>
       </c>
       <c r="C92" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D92" t="s">
         <v>40</v>
@@ -9669,7 +9669,7 @@
         <v>30</v>
       </c>
       <c r="D11" t="s">
-        <v>234</v>
+        <v>30</v>
       </c>
       <c r="E11" t="s">
         <v>30</v>
@@ -10266,7 +10266,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -10385,7 +10385,7 @@
         <v>744</v>
       </c>
       <c r="B13" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C13" t="s">
         <v>908</v>
@@ -10399,7 +10399,7 @@
         <v>744</v>
       </c>
       <c r="B14" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C14" t="s">
         <v>909</v>
@@ -10413,7 +10413,7 @@
         <v>748</v>
       </c>
       <c r="B15" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C15" t="s">
         <v>909</v>
@@ -10427,7 +10427,7 @@
         <v>748</v>
       </c>
       <c r="B16" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C16" t="s">
         <v>910</v>
@@ -10441,7 +10441,7 @@
         <v>752</v>
       </c>
       <c r="B17" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C17" t="s">
         <v>910</v>
@@ -10455,7 +10455,7 @@
         <v>752</v>
       </c>
       <c r="B18" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C18" t="s">
         <v>911</v>
@@ -10469,7 +10469,7 @@
         <v>756</v>
       </c>
       <c r="B19" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C19" t="s">
         <v>911</v>
@@ -10483,7 +10483,7 @@
         <v>756</v>
       </c>
       <c r="B20" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C20" t="s">
         <v>912</v>
@@ -10497,7 +10497,7 @@
         <v>760</v>
       </c>
       <c r="B21" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C21" t="s">
         <v>912</v>
@@ -10511,7 +10511,7 @@
         <v>760</v>
       </c>
       <c r="B22" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C22" t="s">
         <v>913</v>
@@ -10525,7 +10525,7 @@
         <v>764</v>
       </c>
       <c r="B23" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C23" t="s">
         <v>913</v>
@@ -10539,7 +10539,7 @@
         <v>764</v>
       </c>
       <c r="B24" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C24" t="s">
         <v>448</v>
@@ -10553,7 +10553,7 @@
         <v>768</v>
       </c>
       <c r="B25" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C25" t="s">
         <v>448</v>
@@ -10567,7 +10567,7 @@
         <v>768</v>
       </c>
       <c r="B26" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C26" t="s">
         <v>449</v>
@@ -10581,7 +10581,7 @@
         <v>772</v>
       </c>
       <c r="B27" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C27" t="s">
         <v>449</v>
@@ -10595,7 +10595,7 @@
         <v>772</v>
       </c>
       <c r="B28" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C28" t="s">
         <v>450</v>
@@ -10609,7 +10609,7 @@
         <v>776</v>
       </c>
       <c r="B29" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C29" t="s">
         <v>450</v>
@@ -10623,7 +10623,7 @@
         <v>776</v>
       </c>
       <c r="B30" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C30" t="s">
         <v>451</v>
@@ -10637,7 +10637,7 @@
         <v>780</v>
       </c>
       <c r="B31" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C31" t="s">
         <v>451</v>
@@ -10651,7 +10651,7 @@
         <v>780</v>
       </c>
       <c r="B32" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C32" t="s">
         <v>452</v>
@@ -10665,7 +10665,7 @@
         <v>784</v>
       </c>
       <c r="B33" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C33" t="s">
         <v>452</v>
@@ -10679,7 +10679,7 @@
         <v>784</v>
       </c>
       <c r="B34" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C34" t="s">
         <v>453</v>
@@ -10693,7 +10693,7 @@
         <v>788</v>
       </c>
       <c r="B35" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C35" t="s">
         <v>453</v>
@@ -10707,7 +10707,7 @@
         <v>788</v>
       </c>
       <c r="B36" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C36" t="s">
         <v>454</v>
@@ -10721,7 +10721,7 @@
         <v>792</v>
       </c>
       <c r="B37" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C37" t="s">
         <v>454</v>
@@ -10735,7 +10735,7 @@
         <v>792</v>
       </c>
       <c r="B38" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C38" t="s">
         <v>455</v>
@@ -10749,7 +10749,7 @@
         <v>796</v>
       </c>
       <c r="B39" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C39" t="s">
         <v>455</v>
@@ -10763,7 +10763,7 @@
         <v>796</v>
       </c>
       <c r="B40" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C40" t="s">
         <v>456</v>
@@ -10777,7 +10777,7 @@
         <v>800</v>
       </c>
       <c r="B41" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C41" t="s">
         <v>456</v>
@@ -10791,7 +10791,7 @@
         <v>800</v>
       </c>
       <c r="B42" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C42" t="s">
         <v>457</v>
@@ -10805,7 +10805,7 @@
         <v>804</v>
       </c>
       <c r="B43" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C43" t="s">
         <v>457</v>
@@ -10819,7 +10819,7 @@
         <v>804</v>
       </c>
       <c r="B44" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C44" t="s">
         <v>458</v>
@@ -10833,7 +10833,7 @@
         <v>808</v>
       </c>
       <c r="B45" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C45" t="s">
         <v>458</v>
@@ -10847,7 +10847,7 @@
         <v>808</v>
       </c>
       <c r="B46" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C46" t="s">
         <v>459</v>
@@ -10861,7 +10861,7 @@
         <v>812</v>
       </c>
       <c r="B47" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C47" t="s">
         <v>459</v>
@@ -10875,7 +10875,7 @@
         <v>812</v>
       </c>
       <c r="B48" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C48" t="s">
         <v>460</v>
@@ -10889,7 +10889,7 @@
         <v>816</v>
       </c>
       <c r="B49" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C49" t="s">
         <v>460</v>
@@ -10903,7 +10903,7 @@
         <v>816</v>
       </c>
       <c r="B50" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C50" t="s">
         <v>461</v>
@@ -10917,7 +10917,7 @@
         <v>820</v>
       </c>
       <c r="B51" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C51" t="s">
         <v>461</v>
@@ -10931,7 +10931,7 @@
         <v>820</v>
       </c>
       <c r="B52" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C52" t="s">
         <v>462</v>
@@ -10945,7 +10945,7 @@
         <v>824</v>
       </c>
       <c r="B53" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C53" t="s">
         <v>462</v>
@@ -10959,7 +10959,7 @@
         <v>824</v>
       </c>
       <c r="B54" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C54" t="s">
         <v>463</v>
@@ -10973,7 +10973,7 @@
         <v>828</v>
       </c>
       <c r="B55" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C55" t="s">
         <v>463</v>
@@ -10987,7 +10987,7 @@
         <v>828</v>
       </c>
       <c r="B56" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C56" t="s">
         <v>464</v>
@@ -11001,7 +11001,7 @@
         <v>832</v>
       </c>
       <c r="B57" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C57" t="s">
         <v>464</v>
@@ -11015,7 +11015,7 @@
         <v>832</v>
       </c>
       <c r="B58" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C58" t="s">
         <v>465</v>
@@ -11029,7 +11029,7 @@
         <v>836</v>
       </c>
       <c r="B59" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C59" t="s">
         <v>465</v>
@@ -11043,7 +11043,7 @@
         <v>836</v>
       </c>
       <c r="B60" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C60" t="s">
         <v>466</v>
@@ -11057,7 +11057,7 @@
         <v>840</v>
       </c>
       <c r="B61" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C61" t="s">
         <v>466</v>
@@ -11071,7 +11071,7 @@
         <v>840</v>
       </c>
       <c r="B62" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C62" t="s">
         <v>467</v>
@@ -11085,7 +11085,7 @@
         <v>844</v>
       </c>
       <c r="B63" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C63" t="s">
         <v>467</v>
@@ -11099,7 +11099,7 @@
         <v>844</v>
       </c>
       <c r="B64" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C64" t="s">
         <v>468</v>
@@ -11113,7 +11113,7 @@
         <v>848</v>
       </c>
       <c r="B65" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C65" t="s">
         <v>468</v>
@@ -11127,7 +11127,7 @@
         <v>848</v>
       </c>
       <c r="B66" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C66" t="s">
         <v>469</v>
@@ -11141,7 +11141,7 @@
         <v>852</v>
       </c>
       <c r="B67" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C67" t="s">
         <v>469</v>
@@ -11155,7 +11155,7 @@
         <v>852</v>
       </c>
       <c r="B68" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C68" t="s">
         <v>914</v>
@@ -11169,7 +11169,7 @@
         <v>856</v>
       </c>
       <c r="B69" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C69" t="s">
         <v>914</v>
@@ -11183,7 +11183,7 @@
         <v>856</v>
       </c>
       <c r="B70" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C70" t="s">
         <v>915</v>
@@ -11197,7 +11197,7 @@
         <v>860</v>
       </c>
       <c r="B71" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C71" t="s">
         <v>915</v>
@@ -11211,7 +11211,7 @@
         <v>860</v>
       </c>
       <c r="B72" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C72" t="s">
         <v>916</v>
@@ -11225,7 +11225,7 @@
         <v>864</v>
       </c>
       <c r="B73" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C73" t="s">
         <v>916</v>
@@ -11239,7 +11239,7 @@
         <v>864</v>
       </c>
       <c r="B74" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C74" t="s">
         <v>917</v>
@@ -11253,7 +11253,7 @@
         <v>868</v>
       </c>
       <c r="B75" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C75" t="s">
         <v>917</v>
@@ -11267,7 +11267,7 @@
         <v>868</v>
       </c>
       <c r="B76" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C76" t="s">
         <v>918</v>
@@ -11281,7 +11281,7 @@
         <v>872</v>
       </c>
       <c r="B77" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C77" t="s">
         <v>918</v>
@@ -11295,7 +11295,7 @@
         <v>872</v>
       </c>
       <c r="B78" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C78" t="s">
         <v>919</v>
@@ -11309,7 +11309,7 @@
         <v>876</v>
       </c>
       <c r="B79" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C79" t="s">
         <v>919</v>
@@ -11323,7 +11323,7 @@
         <v>876</v>
       </c>
       <c r="B80" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C80" t="s">
         <v>920</v>
@@ -11337,7 +11337,7 @@
         <v>880</v>
       </c>
       <c r="B81" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C81" t="s">
         <v>920</v>
@@ -11351,7 +11351,7 @@
         <v>880</v>
       </c>
       <c r="B82" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C82" t="s">
         <v>921</v>
@@ -11365,7 +11365,7 @@
         <v>884</v>
       </c>
       <c r="B83" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C83" t="s">
         <v>921</v>
@@ -11379,7 +11379,7 @@
         <v>884</v>
       </c>
       <c r="B84" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C84" t="s">
         <v>922</v>
@@ -11393,7 +11393,7 @@
         <v>888</v>
       </c>
       <c r="B85" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C85" t="s">
         <v>922</v>
@@ -11407,7 +11407,7 @@
         <v>888</v>
       </c>
       <c r="B86" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C86" t="s">
         <v>923</v>
@@ -11421,7 +11421,7 @@
         <v>892</v>
       </c>
       <c r="B87" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C87" t="s">
         <v>923</v>
@@ -11435,7 +11435,7 @@
         <v>892</v>
       </c>
       <c r="B88" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C88" t="s">
         <v>924</v>
@@ -11449,7 +11449,7 @@
         <v>896</v>
       </c>
       <c r="B89" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C89" t="s">
         <v>924</v>
@@ -11463,7 +11463,7 @@
         <v>896</v>
       </c>
       <c r="B90" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C90" t="s">
         <v>925</v>
@@ -11477,7 +11477,7 @@
         <v>900</v>
       </c>
       <c r="B91" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C91" t="s">
         <v>925</v>
@@ -11491,7 +11491,7 @@
         <v>900</v>
       </c>
       <c r="B92" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C92" t="s">
         <v>926</v>

</xml_diff>

<commit_message>
refactor(schema)!: derive table keys from table config
</commit_message>
<xml_diff>
--- a/examples/showcase/data/Battle.xlsx
+++ b/examples/showcase/data/Battle.xlsx
@@ -617,7 +617,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -2136,12 +2136,12 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+  <legacyDrawing r:id="anysvml"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -2203,7 +2203,7 @@
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>b0a9bd963cf8bc87</t>
+          <t>d1401fb77a0a2d00</t>
         </is>
       </c>
     </row>
@@ -2333,7 +2333,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>required</t>
+          <t>required;parser=json</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -2575,12 +2575,12 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+  <legacyDrawing r:id="anysvml"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -2644,7 +2644,7 @@
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>996fe1623cec07ee</t>
+          <t>34322ffa4454335d</t>
         </is>
       </c>
     </row>
@@ -2849,7 +2849,7 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>required</t>
+          <t>required;parser=json</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -3619,7 +3619,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+  <legacyDrawing r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -7758,7 +7758,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -10590,7 +10590,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+  <legacyDrawing r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -10658,7 +10658,7 @@
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>18e482d6eedb4d5c</t>
+          <t>fd0a7a4819717e3b</t>
         </is>
       </c>
     </row>
@@ -10808,17 +10808,17 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
+          <t>required;parser=json</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
           <t>required</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>required</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>optional</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add view-based export contracts
</commit_message>
<xml_diff>
--- a/examples/showcase/data/Battle.xlsx
+++ b/examples/showcase/data/Battle.xlsx
@@ -52,7 +52,7 @@
 Tuple cost, e.g. Gold,0,150
 Field: cost
 Type: struct&lt;ResourceCost&gt;
-Scope: all
+Groups: common
 Tuple fields: kind: enum&lt;ResourceKind&gt;, id: i32, count: i32
 Parser: tuple</t>
         </r>
@@ -81,7 +81,7 @@
 JSON object with element/power/radius
 Field: effect
 Type: struct&lt;SkillEffect&gt;
-Scope: all</t>
+Groups: common</t>
         </r>
       </text>
     </comment>
@@ -108,7 +108,7 @@
 Optional item requirement
 Field: required_item
 Type: optional&lt;ref&lt;Item.id&gt;&gt;
-Scope: all</t>
+Groups: common</t>
         </r>
       </text>
     </comment>
@@ -134,7 +134,7 @@
           <t xml:space="preserve">
 Field: cast_origin
 Type: struct&lt;Vec3&gt;
-Scope: all
+Groups: common
 Tuple fields: x: f32, y: f32, z: f32
 Parser: tuple</t>
         </r>
@@ -173,7 +173,7 @@
           <t xml:space="preserve">
 Field: spawn_pos
 Type: struct&lt;Vec3&gt;
-Scope: all
+Groups: common
 Tuple fields: x: f32, y: f32, z: f32
 Parser: tuple</t>
         </r>
@@ -212,7 +212,7 @@
           <t xml:space="preserve">
 Field: spawn_pos
 Type: struct&lt;Vec3&gt;
-Scope: all
+Groups: common
 Tuple fields: x: f32, y: f32, z: f32
 Parser: tuple</t>
         </r>
@@ -251,7 +251,7 @@
           <t xml:space="preserve">
 Field: entry_cost
 Type: struct&lt;ResourceCost&gt;
-Scope: all
+Groups: common
 Tuple fields: kind: enum&lt;ResourceKind&gt;, id: i32, count: i32
 Parser: tuple</t>
         </r>
@@ -282,16 +282,16 @@
     <t>id</t>
   </si>
   <si>
-    <t>@scope</t>
-  </si>
-  <si>
-    <t>all</t>
+    <t>@groups</t>
+  </si>
+  <si>
+    <t>common</t>
   </si>
   <si>
     <t>@schema</t>
   </si>
   <si>
-    <t>70fc913f3e9b878f</t>
+    <t>c894d28c219e5edf</t>
   </si>
   <si>
     <t>#name</t>
@@ -345,7 +345,7 @@
     <t>struct&lt;Vec3&gt;(x: f32, y: f32, z: f32)</t>
   </si>
   <si>
-    <t>#scope</t>
+    <t>#groups</t>
   </si>
   <si>
     <t>#input</t>
@@ -933,7 +933,7 @@
     <t>Character</t>
   </si>
   <si>
-    <t>34322ffa4454335d</t>
+    <t>2553615d93d56167</t>
   </si>
   <si>
     <t>rarity</t>
@@ -1230,7 +1230,7 @@
     <t>list</t>
   </si>
   <si>
-    <t>e92c79afa1e2e40b</t>
+    <t>e0e7445fb45c9c11</t>
   </si>
   <si>
     <t>character_id</t>
@@ -1251,7 +1251,7 @@
     <t>Buff</t>
   </si>
   <si>
-    <t>0b98849d3da9e5fb</t>
+    <t>a50d4c4ce4dfbd8f</t>
   </si>
   <si>
     <t>duration</t>
@@ -1473,7 +1473,7 @@
     <t>DropGroup</t>
   </si>
   <si>
-    <t>ddc8f184c6f4ca0b</t>
+    <t>6d78cabfe88d410d</t>
   </si>
   <si>
     <t>7001</t>
@@ -1599,7 +1599,7 @@
     <t>DropEntry</t>
   </si>
   <si>
-    <t>38e6bc608bd50c74</t>
+    <t>c220c766ac682968</t>
   </si>
   <si>
     <t>group_id</t>
@@ -1701,7 +1701,7 @@
     <t>Monster</t>
   </si>
   <si>
-    <t>3f0a6c4362bc5a57</t>
+    <t>a0b5c7b502b4ed6b</t>
   </si>
   <si>
     <t>level</t>
@@ -2502,7 +2502,7 @@
     <t>Stage</t>
   </si>
   <si>
-    <t>fd0a7a4819717e3b</t>
+    <t>9017b2a46b1a7899</t>
   </si>
   <si>
     <t>monster_ids</t>
@@ -3012,7 +3012,7 @@
     <t>StageReward</t>
   </si>
   <si>
-    <t>0c97ec70735264e3</t>
+    <t>6229c8bb1b11ec13</t>
   </si>
   <si>
     <t>stage_id</t>
@@ -3081,7 +3081,7 @@
     <t>Dungeon</t>
   </si>
   <si>
-    <t>d1401fb77a0a2d00</t>
+    <t>b940457777e98b6c</t>
   </si>
   <si>
     <t>stage_ids</t>

</xml_diff>